<commit_message>
chore: prepare blueprint bundle for public release
</commit_message>
<xml_diff>
--- a/examples/sample_course__blueprint_bundle/sample_course__course_activities.xlsx
+++ b/examples/sample_course__blueprint_bundle/sample_course__course_activities.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P2"/>
+  <dimension ref="A1:P5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -517,10 +517,14 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>CODE-F1</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr"/>
+          <t>CODE-A1</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>file</t>
+        </is>
+      </c>
       <c r="E2" t="inlineStr">
         <is>
           <t>20</t>
@@ -528,7 +532,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>CODE-G1</t>
+          <t>CODE-G-A1</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -541,14 +545,22 @@
           <t>20</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr"/>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>RUB-1: Planning Memo Rubric</t>
+        </is>
+      </c>
       <c r="J2" t="inlineStr">
         <is>
           <t>2026-09-20T03:59:59</t>
         </is>
       </c>
       <c r="K2" t="inlineStr"/>
-      <c r="L2" t="inlineStr"/>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>COND-OPEN</t>
+        </is>
+      </c>
       <c r="M2" t="n">
         <v>1</v>
       </c>
@@ -557,12 +569,198 @@
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>Draft a short planning memo.</t>
+          <t>Draft a short planning memo that names the evidence files you inspected. Use one paragraph for the manifest evidence. Use one paragraph for the activity join evidence.</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>&lt;p&gt;Draft a short planning memo.&lt;/p&gt;</t>
+          <t>&lt;p&gt;Draft a short planning memo that names the evidence files you inspected.&lt;/p&gt;&lt;ul&gt;&lt;li&gt;Use one paragraph for the manifest evidence.&lt;/li&gt;&lt;li&gt;Use one paragraph for the activity join evidence.&lt;/li&gt;&lt;/ul&gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Data Snapshot Worksheet</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>CODE-A2</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>file</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>CODE-G-A2</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Data Snapshot Worksheet</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr"/>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr"/>
+      <c r="L3" t="inlineStr"/>
+      <c r="M3" t="n">
+        <v>1</v>
+      </c>
+      <c r="N3" t="n">
+        <v>0</v>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>Complete the worksheet using the course activities workbook generated by the bundle.</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;Complete the worksheet using the course activities workbook generated by the bundle.&lt;/p&gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Reflection Journal</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>CODE-A3</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>CODE-G-A3</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Reflection Journal</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr"/>
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr"/>
+      <c r="L4" t="inlineStr"/>
+      <c r="M4" t="n">
+        <v>1</v>
+      </c>
+      <c r="N4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>Write a short reflection after reviewing Week 2 materials.</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;Write a short reflection after reviewing Week 2 materials.&lt;/p&gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Unplaced Capstone Draft</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>CODE-AU</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>file</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>CODE-G-AU</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Unplaced Capstone Draft</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr"/>
+      <c r="J5" t="inlineStr"/>
+      <c r="K5" t="inlineStr"/>
+      <c r="L5" t="inlineStr"/>
+      <c r="M5" t="n">
+        <v>0</v>
+      </c>
+      <c r="N5" t="n">
+        <v>0</v>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>This assignment is not linked in the manifest and should appear as unplaced.</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;This assignment is not linked in the manifest and should appear as unplaced.&lt;/p&gt;</t>
         </is>
       </c>
     </row>
@@ -577,7 +775,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R3"/>
+  <dimension ref="A1:R5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -703,7 +901,11 @@
       <c r="H2" t="inlineStr"/>
       <c r="I2" t="inlineStr"/>
       <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr"/>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="inlineStr"/>
       <c r="N2" t="inlineStr"/>
@@ -744,16 +946,40 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>CODE-T1</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr"/>
-      <c r="H3" t="inlineStr"/>
-      <c r="I3" t="inlineStr"/>
+          <t>CODE-D1</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>CODE-G-D1</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Planning Assumptions</t>
+        </is>
+      </c>
       <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr"/>
-      <c r="L3" t="inlineStr"/>
-      <c r="M3" t="inlineStr"/>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="N3" t="inlineStr"/>
       <c r="O3" t="n">
         <v>1</v>
@@ -763,12 +989,160 @@
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>Post one assumption you bring into the course.</t>
+          <t>Post one assumption you bring into source-traceable course review.</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>&lt;p&gt;Post one assumption you bring into the course.&lt;/p&gt;</t>
+          <t>&lt;p&gt;Post one assumption you bring into source-traceable course review.&lt;/p&gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>topic</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>discussion_d2l_1.xml</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>22</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Peer Reply</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>CODE-D2</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>CODE-G-D2</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Peer Reply</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr"/>
+      <c r="O4" t="n">
+        <v>1</v>
+      </c>
+      <c r="P4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>Reply to a peer and identify one item that should remain marked for review.</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;Reply to a peer and identify one item that should remain marked for review.&lt;/p&gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>topic</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>discussion_d2l_1.xml</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Unplaced Help Forum</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>CODE-DU</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr"/>
+      <c r="H5" t="inlineStr"/>
+      <c r="I5" t="inlineStr"/>
+      <c r="J5" t="inlineStr"/>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr"/>
+      <c r="O5" t="n">
+        <v>0</v>
+      </c>
+      <c r="P5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>This discussion topic is not linked in the manifest and should be reported as unplaced.</t>
+        </is>
+      </c>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;This discussion topic is not linked in the manifest and should be reported as unplaced.&lt;/p&gt;</t>
         </is>
       </c>
     </row>
@@ -783,7 +1157,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M2"/>
+  <dimension ref="A1:M9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -866,7 +1240,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>CODE-G1</t>
+          <t>CODE-G-A1</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -882,7 +1256,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>True</t>
+          <t>true</t>
         </is>
       </c>
       <c r="H2" t="inlineStr"/>
@@ -903,6 +1277,359 @@
           <t>dropbox_folder: Planning Memo</t>
         </is>
       </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>9002</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>CODE-G-A2</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Data Snapshot Worksheet</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr"/>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr"/>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr"/>
+      <c r="L3" t="inlineStr"/>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>dropbox_folder: Data Snapshot Worksheet</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>9003</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>CODE-G-A3</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Reflection Journal</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr"/>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr"/>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr"/>
+      <c r="L4" t="inlineStr"/>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>dropbox_folder: Reflection Journal</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>9004</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>CODE-G-Q1</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Readiness Quiz</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr"/>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr"/>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr"/>
+      <c r="L5" t="inlineStr"/>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>quiz: Readiness Quiz</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>9005</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>CODE-G-D1</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Planning Assumptions</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr"/>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr"/>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr"/>
+      <c r="L6" t="inlineStr"/>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>discussion_topic: Planning Assumptions</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>9006</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>CODE-G-D2</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Peer Reply</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr"/>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr"/>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr"/>
+      <c r="L7" t="inlineStr"/>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>discussion_topic: Peer Reply</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>9007</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>CODE-G-AU</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Unplaced Capstone Draft</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr"/>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr"/>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr"/>
+      <c r="L8" t="inlineStr"/>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>dropbox_folder: Unplaced Capstone Draft</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>9008</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>CODE-G-ORPHAN</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Standalone Participation</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr"/>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr"/>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr"/>
+      <c r="L9" t="inlineStr"/>
+      <c r="M9" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -915,7 +1642,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E1"/>
+  <dimension ref="A1:E2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -943,6 +1670,29 @@
         <is>
           <t>quicklink_count</t>
         </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Week 1 Checklist</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>CODE-CL1</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>3</v>
+      </c>
+      <c r="E2" t="n">
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -956,7 +1706,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W1"/>
+  <dimension ref="A1:W2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1073,6 +1823,101 @@
       <c r="W1" t="inlineStr">
         <is>
           <t>instructions_html</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>quiz_d2l_100.xml</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr"/>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>QUIZ-READY</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Readiness Quiz</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>CODE-Q1</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>CODE-G-Q1</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Readiness Quiz</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr"/>
+      <c r="P2" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q2" t="n">
+        <v>3</v>
+      </c>
+      <c r="R2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S2" t="inlineStr"/>
+      <c r="T2" t="n">
+        <v>1</v>
+      </c>
+      <c r="U2" t="n">
+        <v>0</v>
+      </c>
+      <c r="V2" t="inlineStr">
+        <is>
+          <t>Complete this short readiness check after reviewing the Week 1 materials. One attempt is allowed. Questions are drawn from a small pool.</t>
+        </is>
+      </c>
+      <c r="W2" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;Complete this short readiness check after reviewing the Week 1 materials.&lt;/p&gt;&lt;ul&gt;&lt;li&gt;One attempt is allowed.&lt;/li&gt;&lt;li&gt;Questions are drawn from a small pool.&lt;/li&gt;&lt;/ul&gt;</t>
         </is>
       </c>
     </row>
@@ -1087,7 +1932,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F4"/>
+  <dimension ref="A1:F20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1135,7 +1980,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>CODE-F1</t>
+          <t>CODE-A1</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -1145,7 +1990,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>CODE-G1</t>
+          <t>CODE-G-A1</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -1167,17 +2012,17 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>CODE-F1</t>
+          <t>CODE-A1</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>manifest_quicklink</t>
+          <t>rubric</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>1 link(s)</t>
+          <t>RUB-1</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -1189,32 +2034,544 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
+          <t>dropbox_folder</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Planning Memo</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>CODE-A1</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>condition_set</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>COND-OPEN</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>dropbox_folder</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Planning Memo</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>CODE-A1</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>manifest_quicklink</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>1 link(s)</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>dropbox_folder</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Data Snapshot Worksheet</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>CODE-A2</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>grade_item</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>CODE-G-A2</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>dropbox_folder</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Data Snapshot Worksheet</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>CODE-A2</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>manifest_quicklink</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>1 link(s)</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>dropbox_folder</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Reflection Journal</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>CODE-A3</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>grade_item</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>CODE-G-A3</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>dropbox_folder</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Reflection Journal</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>CODE-A3</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>manifest_quicklink</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>1 link(s)</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>dropbox_folder</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Unplaced Capstone Draft</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>CODE-AU</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>grade_item</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>CODE-G-AU</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>dropbox_folder</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Unplaced Capstone Draft</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>CODE-AU</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>manifest_quicklink</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>0 link(s)</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
           <t>discussion_topic</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B12" t="inlineStr">
         <is>
           <t>Planning Assumptions</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>CODE-T1</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>CODE-D1</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>grade_item</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>CODE-G-D1</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>discussion_topic</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Planning Assumptions</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>CODE-D1</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
         <is>
           <t>manifest_quicklink</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="E13" t="inlineStr">
         <is>
           <t>1 link(s)</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="F13" t="inlineStr">
         <is>
           <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>discussion_topic</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Peer Reply</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>CODE-D2</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>grade_item</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>CODE-G-D2</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>discussion_topic</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Peer Reply</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>CODE-D2</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>manifest_quicklink</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>1 link(s)</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>discussion_topic</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Unplaced Help Forum</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>CODE-DU</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>manifest_quicklink</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>0 link(s)</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>checklist</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Week 1 Checklist</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>CODE-CL1</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>manifest_quicklink</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>1 link(s)</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>quiz</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Readiness Quiz</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>CODE-Q1</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>grade_item</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>CODE-G-Q1</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>quiz</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Readiness Quiz</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>CODE-Q1</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>manifest_quicklink</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>1 link(s)</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>grade_item</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Standalone Participation</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>CODE-G-ORPHAN</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>linked_activity</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>(none found in dropbox/discussions/quizzes)</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>none</t>
         </is>
       </c>
     </row>

</xml_diff>